<commit_message>
rm extension binding information 04b9b40658f864ee7c7c7b96cfa351cced5d88f4
</commit_message>
<xml_diff>
--- a/ig/nr-cleaning/StructureDefinition-fr-core-patient-ins.xlsx
+++ b/ig/nr-cleaning/StructureDefinition-fr-core-patient-ins.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7732" uniqueCount="942">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6910" uniqueCount="861">
   <si>
     <t>Property</t>
   </si>
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2023-11-17T10:19:41+00:00</t>
+    <t>2023-11-20T14:22:41+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -2400,265 +2400,22 @@
     <t>RolePerson</t>
   </si>
   <si>
-    <t>The nature of the relationship. Rôle de la personne</t>
+    <t>The nature of the relationship. Rôle de la personne. Ex : personne de confiance, aidant ...</t>
   </si>
   <si>
     <t>https://hl7.fr/ig/fhir/core/ValueSet/fr-core-related-person-role</t>
   </si>
   <si>
-    <t>Patient.contact.relationship:RolePerson.id</t>
-  </si>
-  <si>
-    <t>Patient.contact.relationship.id</t>
-  </si>
-  <si>
-    <t>Patient.contact.relationship:RolePerson.extension</t>
-  </si>
-  <si>
-    <t>Patient.contact.relationship.extension</t>
-  </si>
-  <si>
-    <t>Patient.contact.relationship:RolePerson.coding</t>
-  </si>
-  <si>
-    <t>Patient.contact.relationship.coding</t>
-  </si>
-  <si>
-    <t>Code defined by a terminology system</t>
-  </si>
-  <si>
-    <t>A reference to a code defined by a terminology system.</t>
-  </si>
-  <si>
-    <t>Codes may be defined very casually in enumerations, or code lists, up to very formal definitions such as SNOMED CT - see the HL7 v3 Core Principles for more information.  Ordering of codings is undefined and SHALL NOT be used to infer meaning. Generally, at most only one of the coding values will be labeled as UserSelected = true.</t>
-  </si>
-  <si>
-    <t>Allows for alternative encodings within a code system, and translations to other code systems.</t>
-  </si>
-  <si>
-    <t>CodeableConcept.coding</t>
-  </si>
-  <si>
-    <t>union(., ./translation)</t>
-  </si>
-  <si>
-    <t>C*E.1-8, C*E.10-22</t>
-  </si>
-  <si>
-    <t>Patient.contact.relationship:RolePerson.coding.id</t>
-  </si>
-  <si>
-    <t>Patient.contact.relationship.coding.id</t>
-  </si>
-  <si>
-    <t>Patient.contact.relationship:RolePerson.coding.extension</t>
-  </si>
-  <si>
-    <t>Patient.contact.relationship.coding.extension</t>
-  </si>
-  <si>
-    <t>Patient.contact.relationship:RolePerson.coding.system</t>
-  </si>
-  <si>
-    <t>Patient.contact.relationship.coding.system</t>
-  </si>
-  <si>
-    <t>Identity of the terminology system</t>
-  </si>
-  <si>
-    <t>The identification of the code system that defines the meaning of the symbol in the code.</t>
-  </si>
-  <si>
-    <t>The URI may be an OID (urn:oid:...) or a UUID (urn:uuid:...).  OIDs and UUIDs SHALL be references to the HL7 OID registry. Otherwise, the URI should come from HL7's list of FHIR defined special URIs or it should reference to some definition that establishes the system clearly and unambiguously.</t>
-  </si>
-  <si>
-    <t>Need to be unambiguous about the source of the definition of the symbol.</t>
-  </si>
-  <si>
-    <t>https://mos.esante.gouv.fr/NOS/TRE_R260-HL7RoleClass/FHIR/TRE-R260-HL7RoleClass</t>
-  </si>
-  <si>
-    <t>Coding.system</t>
-  </si>
-  <si>
-    <t>./codeSystem</t>
-  </si>
-  <si>
-    <t>C*E.3</t>
-  </si>
-  <si>
-    <t>Patient.contact.relationship:RolePerson.coding.version</t>
-  </si>
-  <si>
-    <t>Patient.contact.relationship.coding.version</t>
-  </si>
-  <si>
-    <t>Version of the system - if relevant</t>
-  </si>
-  <si>
-    <t>The version of the code system which was used when choosing this code. Note that a well-maintained code system does not need the version reported, because the meaning of codes is consistent across versions. However this cannot consistently be assured, and when the meaning is not guaranteed to be consistent, the version SHOULD be exchanged.</t>
-  </si>
-  <si>
-    <t>Where the terminology does not clearly define what string should be used to identify code system versions, the recommendation is to use the date (expressed in FHIR date format) on which that version was officially published as the version date.</t>
-  </si>
-  <si>
-    <t>Coding.version</t>
-  </si>
-  <si>
-    <t>./codeSystemVersion</t>
-  </si>
-  <si>
-    <t>C*E.7</t>
-  </si>
-  <si>
-    <t>Patient.contact.relationship:RolePerson.coding.code</t>
-  </si>
-  <si>
-    <t>Patient.contact.relationship.coding.code</t>
-  </si>
-  <si>
-    <t>Symbol in syntax defined by the system</t>
-  </si>
-  <si>
-    <t>A symbol in syntax defined by the system. The symbol may be a predefined code or an expression in a syntax defined by the coding system (e.g. post-coordination).</t>
-  </si>
-  <si>
-    <t>Need to refer to a particular code in the system.</t>
-  </si>
-  <si>
-    <t>Coding.code</t>
-  </si>
-  <si>
-    <t>./code</t>
-  </si>
-  <si>
-    <t>C*E.1</t>
-  </si>
-  <si>
-    <t>Patient.contact.relationship:RolePerson.coding.display</t>
-  </si>
-  <si>
-    <t>Patient.contact.relationship.coding.display</t>
-  </si>
-  <si>
-    <t>Representation defined by the system</t>
-  </si>
-  <si>
-    <t>A representation of the meaning of the code in the system, following the rules of the system.</t>
-  </si>
-  <si>
-    <t>Need to be able to carry a human-readable meaning of the code for readers that do not know  the system.</t>
-  </si>
-  <si>
-    <t>Coding.display</t>
-  </si>
-  <si>
-    <t>CV.displayName</t>
-  </si>
-  <si>
-    <t>C*E.2 - but note this is not well followed</t>
-  </si>
-  <si>
-    <t>Patient.contact.relationship:RolePerson.coding.userSelected</t>
-  </si>
-  <si>
-    <t>Patient.contact.relationship.coding.userSelected</t>
-  </si>
-  <si>
-    <t>If this coding was chosen directly by the user</t>
-  </si>
-  <si>
-    <t>Indicates that this coding was chosen by a user directly - e.g. off a pick list of available items (codes or displays).</t>
-  </si>
-  <si>
-    <t>Amongst a set of alternatives, a directly chosen code is the most appropriate starting point for new translations. There is some ambiguity about what exactly 'directly chosen' implies, and trading partner agreement may be needed to clarify the use of this element and its consequences more completely.</t>
-  </si>
-  <si>
-    <t>This has been identified as a clinical safety criterium - that this exact system/code pair was chosen explicitly, rather than inferred by the system based on some rules or language processing.</t>
-  </si>
-  <si>
-    <t>Coding.userSelected</t>
-  </si>
-  <si>
-    <t>CD.codingRationale</t>
-  </si>
-  <si>
-    <t>Sometimes implied by being first</t>
-  </si>
-  <si>
-    <t>Patient.contact.relationship:RolePerson.text</t>
-  </si>
-  <si>
-    <t>Patient.contact.relationship.text</t>
-  </si>
-  <si>
-    <t>Plain text representation of the concept</t>
-  </si>
-  <si>
-    <t>A human language representation of the concept as seen/selected/uttered by the user who entered the data and/or which represents the intended meaning of the user.</t>
-  </si>
-  <si>
-    <t>Very often the text is the same as a displayName of one of the codings.</t>
-  </si>
-  <si>
-    <t>The codes from the terminologies do not always capture the correct meaning with all the nuances of the human using them, or sometimes there is no appropriate code at all. In these cases, the text is used to capture the full meaning of the source.</t>
-  </si>
-  <si>
-    <t>CodeableConcept.text</t>
-  </si>
-  <si>
-    <t>./originalText[mediaType/code="text/plain"]/data</t>
-  </si>
-  <si>
-    <t>C*E.9. But note many systems use C*E.2 for this</t>
-  </si>
-  <si>
     <t>Patient.contact.relationship:RelatedPerson</t>
   </si>
   <si>
     <t>RelatedPerson</t>
   </si>
   <si>
-    <t>The nature of the relationship. Relation de la personne</t>
+    <t>The nature of the relationship. Relation de la personne. Ex : Mère, époux, enfant ...</t>
   </si>
   <si>
     <t>https://hl7.fr/ig/fhir/core/ValueSet/fr-core-related-person</t>
-  </si>
-  <si>
-    <t>Patient.contact.relationship:RelatedPerson.id</t>
-  </si>
-  <si>
-    <t>Patient.contact.relationship:RelatedPerson.extension</t>
-  </si>
-  <si>
-    <t>Patient.contact.relationship:RelatedPerson.coding</t>
-  </si>
-  <si>
-    <t>Patient.contact.relationship:RelatedPerson.coding.id</t>
-  </si>
-  <si>
-    <t>Patient.contact.relationship:RelatedPerson.coding.extension</t>
-  </si>
-  <si>
-    <t>Patient.contact.relationship:RelatedPerson.coding.system</t>
-  </si>
-  <si>
-    <t>https://mos.esante.gouv.fr/NOS/TRE_R216-HL7RoleCode/FHIR/TRE-R216-HL7RoleCode</t>
-  </si>
-  <si>
-    <t>Patient.contact.relationship:RelatedPerson.coding.version</t>
-  </si>
-  <si>
-    <t>Patient.contact.relationship:RelatedPerson.coding.code</t>
-  </si>
-  <si>
-    <t>Patient.contact.relationship:RelatedPerson.coding.display</t>
-  </si>
-  <si>
-    <t>Patient.contact.relationship:RelatedPerson.coding.userSelected</t>
-  </si>
-  <si>
-    <t>Patient.contact.relationship:RelatedPerson.text</t>
   </si>
   <si>
     <t>Patient.contact.name</t>
@@ -3261,11 +3018,11 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:AO207"/>
+  <dimension ref="A1:AO185"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
     <col min="1" max="1" width="69.5859375" customWidth="true" bestFit="true"/>
-    <col min="2" max="2" width="45.59375" customWidth="true" bestFit="true"/>
+    <col min="2" max="2" width="39.47265625" customWidth="true" bestFit="true"/>
     <col min="3" max="3" width="24.2265625" customWidth="true" bestFit="true" hidden="true"/>
     <col min="4" max="4" width="39.9140625" customWidth="true" bestFit="true" hidden="true"/>
     <col min="5" max="5" width="6.77734375" customWidth="true" bestFit="true"/>
@@ -22533,9 +22290,11 @@
         <v>760</v>
       </c>
       <c r="B165" t="s" s="2">
+        <v>747</v>
+      </c>
+      <c r="C165" t="s" s="2">
         <v>761</v>
       </c>
-      <c r="C165" s="2"/>
       <c r="D165" t="s" s="2">
         <v>79</v>
       </c>
@@ -22556,16 +22315,20 @@
         <v>79</v>
       </c>
       <c r="K165" t="s" s="2">
-        <v>103</v>
+        <v>438</v>
       </c>
       <c r="L165" t="s" s="2">
-        <v>104</v>
+        <v>762</v>
       </c>
       <c r="M165" t="s" s="2">
-        <v>105</v>
-      </c>
-      <c r="N165" s="2"/>
-      <c r="O165" s="2"/>
+        <v>749</v>
+      </c>
+      <c r="N165" t="s" s="2">
+        <v>698</v>
+      </c>
+      <c r="O165" t="s" s="2">
+        <v>750</v>
+      </c>
       <c r="P165" t="s" s="2">
         <v>79</v>
       </c>
@@ -22589,13 +22352,11 @@
         <v>79</v>
       </c>
       <c r="X165" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="Y165" t="s" s="2">
-        <v>79</v>
-      </c>
+        <v>151</v>
+      </c>
+      <c r="Y165" s="2"/>
       <c r="Z165" t="s" s="2">
-        <v>79</v>
+        <v>763</v>
       </c>
       <c r="AA165" t="s" s="2">
         <v>79</v>
@@ -22613,31 +22374,31 @@
         <v>79</v>
       </c>
       <c r="AF165" t="s" s="2">
-        <v>106</v>
+        <v>747</v>
       </c>
       <c r="AG165" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AH165" t="s" s="2">
-        <v>87</v>
+        <v>78</v>
       </c>
       <c r="AI165" t="s" s="2">
-        <v>79</v>
+        <v>99</v>
       </c>
       <c r="AJ165" t="s" s="2">
-        <v>79</v>
+        <v>100</v>
       </c>
       <c r="AK165" t="s" s="2">
+        <v>754</v>
+      </c>
+      <c r="AL165" t="s" s="2">
         <v>107</v>
       </c>
-      <c r="AL165" t="s" s="2">
-        <v>79</v>
-      </c>
       <c r="AM165" t="s" s="2">
         <v>79</v>
       </c>
       <c r="AN165" t="s" s="2">
-        <v>79</v>
+        <v>755</v>
       </c>
       <c r="AO165" t="s" s="2">
         <v>79</v>
@@ -22645,21 +22406,21 @@
     </row>
     <row r="166">
       <c r="A166" t="s" s="2">
-        <v>762</v>
+        <v>764</v>
       </c>
       <c r="B166" t="s" s="2">
-        <v>763</v>
+        <v>764</v>
       </c>
       <c r="C166" s="2"/>
       <c r="D166" t="s" s="2">
-        <v>109</v>
+        <v>79</v>
       </c>
       <c r="E166" s="2"/>
       <c r="F166" t="s" s="2">
         <v>77</v>
       </c>
       <c r="G166" t="s" s="2">
-        <v>78</v>
+        <v>87</v>
       </c>
       <c r="H166" t="s" s="2">
         <v>79</v>
@@ -22671,18 +22432,20 @@
         <v>79</v>
       </c>
       <c r="K166" t="s" s="2">
-        <v>110</v>
+        <v>566</v>
       </c>
       <c r="L166" t="s" s="2">
-        <v>111</v>
+        <v>765</v>
       </c>
       <c r="M166" t="s" s="2">
-        <v>112</v>
+        <v>766</v>
       </c>
       <c r="N166" t="s" s="2">
-        <v>113</v>
-      </c>
-      <c r="O166" s="2"/>
+        <v>767</v>
+      </c>
+      <c r="O166" t="s" s="2">
+        <v>768</v>
+      </c>
       <c r="P166" t="s" s="2">
         <v>79</v>
       </c>
@@ -22718,34 +22481,34 @@
         <v>79</v>
       </c>
       <c r="AB166" t="s" s="2">
-        <v>114</v>
+        <v>79</v>
       </c>
       <c r="AC166" t="s" s="2">
-        <v>115</v>
+        <v>79</v>
       </c>
       <c r="AD166" t="s" s="2">
         <v>79</v>
       </c>
       <c r="AE166" t="s" s="2">
-        <v>116</v>
+        <v>79</v>
       </c>
       <c r="AF166" t="s" s="2">
-        <v>117</v>
+        <v>764</v>
       </c>
       <c r="AG166" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AH166" t="s" s="2">
-        <v>78</v>
+        <v>87</v>
       </c>
       <c r="AI166" t="s" s="2">
         <v>99</v>
       </c>
       <c r="AJ166" t="s" s="2">
-        <v>118</v>
+        <v>100</v>
       </c>
       <c r="AK166" t="s" s="2">
-        <v>101</v>
+        <v>769</v>
       </c>
       <c r="AL166" t="s" s="2">
         <v>79</v>
@@ -22754,7 +22517,7 @@
         <v>79</v>
       </c>
       <c r="AN166" t="s" s="2">
-        <v>79</v>
+        <v>770</v>
       </c>
       <c r="AO166" t="s" s="2">
         <v>79</v>
@@ -22762,10 +22525,10 @@
     </row>
     <row r="167">
       <c r="A167" t="s" s="2">
-        <v>764</v>
+        <v>771</v>
       </c>
       <c r="B167" t="s" s="2">
-        <v>765</v>
+        <v>771</v>
       </c>
       <c r="C167" s="2"/>
       <c r="D167" t="s" s="2">
@@ -22785,22 +22548,22 @@
         <v>79</v>
       </c>
       <c r="J167" t="s" s="2">
-        <v>88</v>
+        <v>79</v>
       </c>
       <c r="K167" t="s" s="2">
-        <v>147</v>
+        <v>660</v>
       </c>
       <c r="L167" t="s" s="2">
-        <v>766</v>
+        <v>661</v>
       </c>
       <c r="M167" t="s" s="2">
-        <v>767</v>
+        <v>662</v>
       </c>
       <c r="N167" t="s" s="2">
-        <v>768</v>
+        <v>772</v>
       </c>
       <c r="O167" t="s" s="2">
-        <v>769</v>
+        <v>664</v>
       </c>
       <c r="P167" t="s" s="2">
         <v>79</v>
@@ -22849,7 +22612,7 @@
         <v>79</v>
       </c>
       <c r="AF167" t="s" s="2">
-        <v>770</v>
+        <v>771</v>
       </c>
       <c r="AG167" t="s" s="2">
         <v>77</v>
@@ -22861,10 +22624,10 @@
         <v>99</v>
       </c>
       <c r="AJ167" t="s" s="2">
-        <v>100</v>
+        <v>665</v>
       </c>
       <c r="AK167" t="s" s="2">
-        <v>771</v>
+        <v>666</v>
       </c>
       <c r="AL167" t="s" s="2">
         <v>79</v>
@@ -22873,7 +22636,7 @@
         <v>79</v>
       </c>
       <c r="AN167" t="s" s="2">
-        <v>772</v>
+        <v>667</v>
       </c>
       <c r="AO167" t="s" s="2">
         <v>79</v>
@@ -22884,7 +22647,7 @@
         <v>773</v>
       </c>
       <c r="B168" t="s" s="2">
-        <v>774</v>
+        <v>773</v>
       </c>
       <c r="C168" s="2"/>
       <c r="D168" t="s" s="2">
@@ -22907,16 +22670,20 @@
         <v>79</v>
       </c>
       <c r="K168" t="s" s="2">
-        <v>103</v>
+        <v>774</v>
       </c>
       <c r="L168" t="s" s="2">
-        <v>104</v>
+        <v>775</v>
       </c>
       <c r="M168" t="s" s="2">
-        <v>105</v>
-      </c>
-      <c r="N168" s="2"/>
-      <c r="O168" s="2"/>
+        <v>776</v>
+      </c>
+      <c r="N168" t="s" s="2">
+        <v>292</v>
+      </c>
+      <c r="O168" t="s" s="2">
+        <v>777</v>
+      </c>
       <c r="P168" t="s" s="2">
         <v>79</v>
       </c>
@@ -22964,7 +22731,7 @@
         <v>79</v>
       </c>
       <c r="AF168" t="s" s="2">
-        <v>106</v>
+        <v>773</v>
       </c>
       <c r="AG168" t="s" s="2">
         <v>77</v>
@@ -22973,22 +22740,22 @@
         <v>87</v>
       </c>
       <c r="AI168" t="s" s="2">
-        <v>79</v>
+        <v>99</v>
       </c>
       <c r="AJ168" t="s" s="2">
-        <v>79</v>
+        <v>100</v>
       </c>
       <c r="AK168" t="s" s="2">
+        <v>778</v>
+      </c>
+      <c r="AL168" t="s" s="2">
         <v>107</v>
       </c>
-      <c r="AL168" t="s" s="2">
-        <v>79</v>
-      </c>
       <c r="AM168" t="s" s="2">
         <v>79</v>
       </c>
       <c r="AN168" t="s" s="2">
-        <v>79</v>
+        <v>779</v>
       </c>
       <c r="AO168" t="s" s="2">
         <v>79</v>
@@ -22996,21 +22763,21 @@
     </row>
     <row r="169">
       <c r="A169" t="s" s="2">
-        <v>775</v>
+        <v>780</v>
       </c>
       <c r="B169" t="s" s="2">
-        <v>776</v>
+        <v>780</v>
       </c>
       <c r="C169" s="2"/>
       <c r="D169" t="s" s="2">
-        <v>109</v>
+        <v>79</v>
       </c>
       <c r="E169" s="2"/>
       <c r="F169" t="s" s="2">
         <v>77</v>
       </c>
       <c r="G169" t="s" s="2">
-        <v>78</v>
+        <v>87</v>
       </c>
       <c r="H169" t="s" s="2">
         <v>79</v>
@@ -23022,18 +22789,20 @@
         <v>79</v>
       </c>
       <c r="K169" t="s" s="2">
-        <v>110</v>
+        <v>171</v>
       </c>
       <c r="L169" t="s" s="2">
-        <v>111</v>
+        <v>781</v>
       </c>
       <c r="M169" t="s" s="2">
-        <v>112</v>
+        <v>782</v>
       </c>
       <c r="N169" t="s" s="2">
-        <v>113</v>
-      </c>
-      <c r="O169" s="2"/>
+        <v>340</v>
+      </c>
+      <c r="O169" t="s" s="2">
+        <v>783</v>
+      </c>
       <c r="P169" t="s" s="2">
         <v>79</v>
       </c>
@@ -23057,55 +22826,55 @@
         <v>79</v>
       </c>
       <c r="X169" t="s" s="2">
-        <v>79</v>
+        <v>262</v>
       </c>
       <c r="Y169" t="s" s="2">
-        <v>79</v>
+        <v>784</v>
       </c>
       <c r="Z169" t="s" s="2">
-        <v>79</v>
+        <v>785</v>
       </c>
       <c r="AA169" t="s" s="2">
         <v>79</v>
       </c>
       <c r="AB169" t="s" s="2">
-        <v>114</v>
+        <v>79</v>
       </c>
       <c r="AC169" t="s" s="2">
-        <v>115</v>
+        <v>79</v>
       </c>
       <c r="AD169" t="s" s="2">
         <v>79</v>
       </c>
       <c r="AE169" t="s" s="2">
-        <v>116</v>
+        <v>79</v>
       </c>
       <c r="AF169" t="s" s="2">
-        <v>117</v>
+        <v>780</v>
       </c>
       <c r="AG169" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AH169" t="s" s="2">
-        <v>78</v>
+        <v>87</v>
       </c>
       <c r="AI169" t="s" s="2">
         <v>99</v>
       </c>
       <c r="AJ169" t="s" s="2">
-        <v>118</v>
+        <v>100</v>
       </c>
       <c r="AK169" t="s" s="2">
-        <v>101</v>
+        <v>674</v>
       </c>
       <c r="AL169" t="s" s="2">
-        <v>79</v>
+        <v>107</v>
       </c>
       <c r="AM169" t="s" s="2">
         <v>79</v>
       </c>
       <c r="AN169" t="s" s="2">
-        <v>79</v>
+        <v>786</v>
       </c>
       <c r="AO169" t="s" s="2">
         <v>79</v>
@@ -23113,10 +22882,10 @@
     </row>
     <row r="170">
       <c r="A170" t="s" s="2">
-        <v>777</v>
+        <v>787</v>
       </c>
       <c r="B170" t="s" s="2">
-        <v>778</v>
+        <v>787</v>
       </c>
       <c r="C170" s="2"/>
       <c r="D170" t="s" s="2">
@@ -23124,7 +22893,7 @@
       </c>
       <c r="E170" s="2"/>
       <c r="F170" t="s" s="2">
-        <v>87</v>
+        <v>77</v>
       </c>
       <c r="G170" t="s" s="2">
         <v>87</v>
@@ -23136,22 +22905,22 @@
         <v>79</v>
       </c>
       <c r="J170" t="s" s="2">
-        <v>88</v>
+        <v>79</v>
       </c>
       <c r="K170" t="s" s="2">
-        <v>131</v>
+        <v>476</v>
       </c>
       <c r="L170" t="s" s="2">
-        <v>779</v>
+        <v>788</v>
       </c>
       <c r="M170" t="s" s="2">
-        <v>780</v>
+        <v>789</v>
       </c>
       <c r="N170" t="s" s="2">
-        <v>781</v>
+        <v>790</v>
       </c>
       <c r="O170" t="s" s="2">
-        <v>782</v>
+        <v>791</v>
       </c>
       <c r="P170" t="s" s="2">
         <v>79</v>
@@ -23161,7 +22930,7 @@
         <v>79</v>
       </c>
       <c r="S170" t="s" s="2">
-        <v>783</v>
+        <v>79</v>
       </c>
       <c r="T170" t="s" s="2">
         <v>79</v>
@@ -23200,7 +22969,7 @@
         <v>79</v>
       </c>
       <c r="AF170" t="s" s="2">
-        <v>784</v>
+        <v>787</v>
       </c>
       <c r="AG170" t="s" s="2">
         <v>77</v>
@@ -23209,22 +22978,22 @@
         <v>87</v>
       </c>
       <c r="AI170" t="s" s="2">
-        <v>99</v>
+        <v>792</v>
       </c>
       <c r="AJ170" t="s" s="2">
-        <v>100</v>
+        <v>481</v>
       </c>
       <c r="AK170" t="s" s="2">
-        <v>785</v>
+        <v>793</v>
       </c>
       <c r="AL170" t="s" s="2">
-        <v>79</v>
+        <v>107</v>
       </c>
       <c r="AM170" t="s" s="2">
         <v>79</v>
       </c>
       <c r="AN170" t="s" s="2">
-        <v>786</v>
+        <v>794</v>
       </c>
       <c r="AO170" t="s" s="2">
         <v>79</v>
@@ -23232,10 +23001,10 @@
     </row>
     <row r="171">
       <c r="A171" t="s" s="2">
-        <v>787</v>
+        <v>795</v>
       </c>
       <c r="B171" t="s" s="2">
-        <v>788</v>
+        <v>795</v>
       </c>
       <c r="C171" s="2"/>
       <c r="D171" t="s" s="2">
@@ -23255,19 +23024,19 @@
         <v>79</v>
       </c>
       <c r="J171" t="s" s="2">
-        <v>88</v>
+        <v>79</v>
       </c>
       <c r="K171" t="s" s="2">
-        <v>103</v>
+        <v>391</v>
       </c>
       <c r="L171" t="s" s="2">
-        <v>789</v>
+        <v>796</v>
       </c>
       <c r="M171" t="s" s="2">
-        <v>790</v>
+        <v>797</v>
       </c>
       <c r="N171" t="s" s="2">
-        <v>791</v>
+        <v>394</v>
       </c>
       <c r="O171" s="2"/>
       <c r="P171" t="s" s="2">
@@ -23317,7 +23086,7 @@
         <v>79</v>
       </c>
       <c r="AF171" t="s" s="2">
-        <v>792</v>
+        <v>795</v>
       </c>
       <c r="AG171" t="s" s="2">
         <v>77</v>
@@ -23329,19 +23098,19 @@
         <v>99</v>
       </c>
       <c r="AJ171" t="s" s="2">
-        <v>100</v>
+        <v>398</v>
       </c>
       <c r="AK171" t="s" s="2">
-        <v>793</v>
+        <v>798</v>
       </c>
       <c r="AL171" t="s" s="2">
-        <v>79</v>
+        <v>107</v>
       </c>
       <c r="AM171" t="s" s="2">
         <v>79</v>
       </c>
       <c r="AN171" t="s" s="2">
-        <v>794</v>
+        <v>799</v>
       </c>
       <c r="AO171" t="s" s="2">
         <v>79</v>
@@ -23349,10 +23118,10 @@
     </row>
     <row r="172">
       <c r="A172" t="s" s="2">
-        <v>795</v>
+        <v>800</v>
       </c>
       <c r="B172" t="s" s="2">
-        <v>796</v>
+        <v>800</v>
       </c>
       <c r="C172" s="2"/>
       <c r="D172" t="s" s="2">
@@ -23363,7 +23132,7 @@
         <v>77</v>
       </c>
       <c r="G172" t="s" s="2">
-        <v>87</v>
+        <v>78</v>
       </c>
       <c r="H172" t="s" s="2">
         <v>79</v>
@@ -23372,22 +23141,22 @@
         <v>79</v>
       </c>
       <c r="J172" t="s" s="2">
-        <v>88</v>
+        <v>79</v>
       </c>
       <c r="K172" t="s" s="2">
-        <v>171</v>
+        <v>723</v>
       </c>
       <c r="L172" t="s" s="2">
-        <v>797</v>
+        <v>801</v>
       </c>
       <c r="M172" t="s" s="2">
-        <v>798</v>
+        <v>802</v>
       </c>
       <c r="N172" t="s" s="2">
-        <v>340</v>
+        <v>803</v>
       </c>
       <c r="O172" t="s" s="2">
-        <v>799</v>
+        <v>804</v>
       </c>
       <c r="P172" t="s" s="2">
         <v>79</v>
@@ -23442,7 +23211,7 @@
         <v>77</v>
       </c>
       <c r="AH172" t="s" s="2">
-        <v>87</v>
+        <v>78</v>
       </c>
       <c r="AI172" t="s" s="2">
         <v>99</v>
@@ -23451,16 +23220,16 @@
         <v>100</v>
       </c>
       <c r="AK172" t="s" s="2">
-        <v>801</v>
+        <v>805</v>
       </c>
       <c r="AL172" t="s" s="2">
-        <v>79</v>
+        <v>806</v>
       </c>
       <c r="AM172" t="s" s="2">
         <v>79</v>
       </c>
       <c r="AN172" t="s" s="2">
-        <v>802</v>
+        <v>79</v>
       </c>
       <c r="AO172" t="s" s="2">
         <v>79</v>
@@ -23468,10 +23237,10 @@
     </row>
     <row r="173">
       <c r="A173" t="s" s="2">
-        <v>803</v>
+        <v>807</v>
       </c>
       <c r="B173" t="s" s="2">
-        <v>804</v>
+        <v>807</v>
       </c>
       <c r="C173" s="2"/>
       <c r="D173" t="s" s="2">
@@ -23491,23 +23260,19 @@
         <v>79</v>
       </c>
       <c r="J173" t="s" s="2">
-        <v>88</v>
+        <v>79</v>
       </c>
       <c r="K173" t="s" s="2">
         <v>103</v>
       </c>
       <c r="L173" t="s" s="2">
-        <v>805</v>
+        <v>104</v>
       </c>
       <c r="M173" t="s" s="2">
-        <v>806</v>
-      </c>
-      <c r="N173" t="s" s="2">
-        <v>340</v>
-      </c>
-      <c r="O173" t="s" s="2">
-        <v>807</v>
-      </c>
+        <v>105</v>
+      </c>
+      <c r="N173" s="2"/>
+      <c r="O173" s="2"/>
       <c r="P173" t="s" s="2">
         <v>79</v>
       </c>
@@ -23555,7 +23320,7 @@
         <v>79</v>
       </c>
       <c r="AF173" t="s" s="2">
-        <v>808</v>
+        <v>106</v>
       </c>
       <c r="AG173" t="s" s="2">
         <v>77</v>
@@ -23564,13 +23329,13 @@
         <v>87</v>
       </c>
       <c r="AI173" t="s" s="2">
-        <v>99</v>
+        <v>79</v>
       </c>
       <c r="AJ173" t="s" s="2">
-        <v>100</v>
+        <v>79</v>
       </c>
       <c r="AK173" t="s" s="2">
-        <v>809</v>
+        <v>107</v>
       </c>
       <c r="AL173" t="s" s="2">
         <v>79</v>
@@ -23579,7 +23344,7 @@
         <v>79</v>
       </c>
       <c r="AN173" t="s" s="2">
-        <v>810</v>
+        <v>79</v>
       </c>
       <c r="AO173" t="s" s="2">
         <v>79</v>
@@ -23587,21 +23352,21 @@
     </row>
     <row r="174">
       <c r="A174" t="s" s="2">
-        <v>811</v>
+        <v>808</v>
       </c>
       <c r="B174" t="s" s="2">
-        <v>812</v>
+        <v>808</v>
       </c>
       <c r="C174" s="2"/>
       <c r="D174" t="s" s="2">
-        <v>79</v>
+        <v>109</v>
       </c>
       <c r="E174" s="2"/>
       <c r="F174" t="s" s="2">
         <v>77</v>
       </c>
       <c r="G174" t="s" s="2">
-        <v>87</v>
+        <v>78</v>
       </c>
       <c r="H174" t="s" s="2">
         <v>79</v>
@@ -23610,23 +23375,21 @@
         <v>79</v>
       </c>
       <c r="J174" t="s" s="2">
-        <v>88</v>
+        <v>79</v>
       </c>
       <c r="K174" t="s" s="2">
-        <v>557</v>
+        <v>110</v>
       </c>
       <c r="L174" t="s" s="2">
-        <v>813</v>
+        <v>111</v>
       </c>
       <c r="M174" t="s" s="2">
-        <v>814</v>
+        <v>112</v>
       </c>
       <c r="N174" t="s" s="2">
-        <v>815</v>
-      </c>
-      <c r="O174" t="s" s="2">
-        <v>816</v>
-      </c>
+        <v>113</v>
+      </c>
+      <c r="O174" s="2"/>
       <c r="P174" t="s" s="2">
         <v>79</v>
       </c>
@@ -23662,34 +23425,34 @@
         <v>79</v>
       </c>
       <c r="AB174" t="s" s="2">
-        <v>79</v>
+        <v>114</v>
       </c>
       <c r="AC174" t="s" s="2">
-        <v>79</v>
+        <v>115</v>
       </c>
       <c r="AD174" t="s" s="2">
         <v>79</v>
       </c>
       <c r="AE174" t="s" s="2">
-        <v>79</v>
+        <v>116</v>
       </c>
       <c r="AF174" t="s" s="2">
-        <v>817</v>
+        <v>117</v>
       </c>
       <c r="AG174" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AH174" t="s" s="2">
-        <v>87</v>
+        <v>78</v>
       </c>
       <c r="AI174" t="s" s="2">
         <v>99</v>
       </c>
       <c r="AJ174" t="s" s="2">
-        <v>100</v>
+        <v>118</v>
       </c>
       <c r="AK174" t="s" s="2">
-        <v>818</v>
+        <v>101</v>
       </c>
       <c r="AL174" t="s" s="2">
         <v>79</v>
@@ -23698,7 +23461,7 @@
         <v>79</v>
       </c>
       <c r="AN174" t="s" s="2">
-        <v>819</v>
+        <v>79</v>
       </c>
       <c r="AO174" t="s" s="2">
         <v>79</v>
@@ -23706,45 +23469,45 @@
     </row>
     <row r="175">
       <c r="A175" t="s" s="2">
-        <v>820</v>
+        <v>809</v>
       </c>
       <c r="B175" t="s" s="2">
-        <v>821</v>
+        <v>809</v>
       </c>
       <c r="C175" s="2"/>
       <c r="D175" t="s" s="2">
-        <v>79</v>
+        <v>743</v>
       </c>
       <c r="E175" s="2"/>
       <c r="F175" t="s" s="2">
         <v>77</v>
       </c>
       <c r="G175" t="s" s="2">
-        <v>87</v>
+        <v>78</v>
       </c>
       <c r="H175" t="s" s="2">
         <v>79</v>
       </c>
       <c r="I175" t="s" s="2">
-        <v>79</v>
+        <v>88</v>
       </c>
       <c r="J175" t="s" s="2">
         <v>88</v>
       </c>
       <c r="K175" t="s" s="2">
-        <v>103</v>
+        <v>110</v>
       </c>
       <c r="L175" t="s" s="2">
-        <v>822</v>
+        <v>744</v>
       </c>
       <c r="M175" t="s" s="2">
-        <v>823</v>
+        <v>745</v>
       </c>
       <c r="N175" t="s" s="2">
-        <v>824</v>
+        <v>113</v>
       </c>
       <c r="O175" t="s" s="2">
-        <v>825</v>
+        <v>404</v>
       </c>
       <c r="P175" t="s" s="2">
         <v>79</v>
@@ -23793,22 +23556,22 @@
         <v>79</v>
       </c>
       <c r="AF175" t="s" s="2">
-        <v>826</v>
+        <v>746</v>
       </c>
       <c r="AG175" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AH175" t="s" s="2">
-        <v>87</v>
+        <v>78</v>
       </c>
       <c r="AI175" t="s" s="2">
         <v>99</v>
       </c>
       <c r="AJ175" t="s" s="2">
-        <v>100</v>
+        <v>118</v>
       </c>
       <c r="AK175" t="s" s="2">
-        <v>827</v>
+        <v>101</v>
       </c>
       <c r="AL175" t="s" s="2">
         <v>79</v>
@@ -23817,7 +23580,7 @@
         <v>79</v>
       </c>
       <c r="AN175" t="s" s="2">
-        <v>828</v>
+        <v>79</v>
       </c>
       <c r="AO175" t="s" s="2">
         <v>79</v>
@@ -23825,20 +23588,18 @@
     </row>
     <row r="176">
       <c r="A176" t="s" s="2">
-        <v>829</v>
+        <v>810</v>
       </c>
       <c r="B176" t="s" s="2">
-        <v>747</v>
-      </c>
-      <c r="C176" t="s" s="2">
-        <v>830</v>
-      </c>
+        <v>810</v>
+      </c>
+      <c r="C176" s="2"/>
       <c r="D176" t="s" s="2">
         <v>79</v>
       </c>
       <c r="E176" s="2"/>
       <c r="F176" t="s" s="2">
-        <v>77</v>
+        <v>87</v>
       </c>
       <c r="G176" t="s" s="2">
         <v>87</v>
@@ -23856,16 +23617,16 @@
         <v>438</v>
       </c>
       <c r="L176" t="s" s="2">
-        <v>831</v>
+        <v>811</v>
       </c>
       <c r="M176" t="s" s="2">
-        <v>749</v>
+        <v>812</v>
       </c>
       <c r="N176" t="s" s="2">
-        <v>698</v>
+        <v>813</v>
       </c>
       <c r="O176" t="s" s="2">
-        <v>750</v>
+        <v>814</v>
       </c>
       <c r="P176" t="s" s="2">
         <v>79</v>
@@ -23890,11 +23651,13 @@
         <v>79</v>
       </c>
       <c r="X176" t="s" s="2">
-        <v>151</v>
-      </c>
-      <c r="Y176" s="2"/>
+        <v>175</v>
+      </c>
+      <c r="Y176" t="s" s="2">
+        <v>176</v>
+      </c>
       <c r="Z176" t="s" s="2">
-        <v>832</v>
+        <v>177</v>
       </c>
       <c r="AA176" t="s" s="2">
         <v>79</v>
@@ -23912,13 +23675,13 @@
         <v>79</v>
       </c>
       <c r="AF176" t="s" s="2">
-        <v>747</v>
+        <v>810</v>
       </c>
       <c r="AG176" t="s" s="2">
-        <v>77</v>
+        <v>87</v>
       </c>
       <c r="AH176" t="s" s="2">
-        <v>78</v>
+        <v>87</v>
       </c>
       <c r="AI176" t="s" s="2">
         <v>99</v>
@@ -23927,16 +23690,16 @@
         <v>100</v>
       </c>
       <c r="AK176" t="s" s="2">
-        <v>754</v>
+        <v>815</v>
       </c>
       <c r="AL176" t="s" s="2">
-        <v>107</v>
+        <v>816</v>
       </c>
       <c r="AM176" t="s" s="2">
         <v>79</v>
       </c>
       <c r="AN176" t="s" s="2">
-        <v>755</v>
+        <v>817</v>
       </c>
       <c r="AO176" t="s" s="2">
         <v>79</v>
@@ -23944,10 +23707,10 @@
     </row>
     <row r="177">
       <c r="A177" t="s" s="2">
-        <v>833</v>
+        <v>818</v>
       </c>
       <c r="B177" t="s" s="2">
-        <v>761</v>
+        <v>818</v>
       </c>
       <c r="C177" s="2"/>
       <c r="D177" t="s" s="2">
@@ -23970,16 +23733,20 @@
         <v>79</v>
       </c>
       <c r="K177" t="s" s="2">
-        <v>103</v>
+        <v>557</v>
       </c>
       <c r="L177" t="s" s="2">
-        <v>104</v>
+        <v>819</v>
       </c>
       <c r="M177" t="s" s="2">
-        <v>105</v>
-      </c>
-      <c r="N177" s="2"/>
-      <c r="O177" s="2"/>
+        <v>820</v>
+      </c>
+      <c r="N177" t="s" s="2">
+        <v>821</v>
+      </c>
+      <c r="O177" t="s" s="2">
+        <v>822</v>
+      </c>
       <c r="P177" t="s" s="2">
         <v>79</v>
       </c>
@@ -24027,7 +23794,7 @@
         <v>79</v>
       </c>
       <c r="AF177" t="s" s="2">
-        <v>106</v>
+        <v>818</v>
       </c>
       <c r="AG177" t="s" s="2">
         <v>77</v>
@@ -24036,22 +23803,22 @@
         <v>87</v>
       </c>
       <c r="AI177" t="s" s="2">
-        <v>79</v>
+        <v>99</v>
       </c>
       <c r="AJ177" t="s" s="2">
-        <v>79</v>
+        <v>100</v>
       </c>
       <c r="AK177" t="s" s="2">
-        <v>107</v>
+        <v>823</v>
       </c>
       <c r="AL177" t="s" s="2">
-        <v>79</v>
+        <v>824</v>
       </c>
       <c r="AM177" t="s" s="2">
         <v>79</v>
       </c>
       <c r="AN177" t="s" s="2">
-        <v>79</v>
+        <v>825</v>
       </c>
       <c r="AO177" t="s" s="2">
         <v>79</v>
@@ -24059,14 +23826,14 @@
     </row>
     <row r="178">
       <c r="A178" t="s" s="2">
-        <v>834</v>
+        <v>826</v>
       </c>
       <c r="B178" t="s" s="2">
-        <v>763</v>
+        <v>826</v>
       </c>
       <c r="C178" s="2"/>
       <c r="D178" t="s" s="2">
-        <v>109</v>
+        <v>827</v>
       </c>
       <c r="E178" s="2"/>
       <c r="F178" t="s" s="2">
@@ -24085,16 +23852,16 @@
         <v>79</v>
       </c>
       <c r="K178" t="s" s="2">
-        <v>110</v>
+        <v>828</v>
       </c>
       <c r="L178" t="s" s="2">
-        <v>111</v>
+        <v>829</v>
       </c>
       <c r="M178" t="s" s="2">
-        <v>112</v>
+        <v>830</v>
       </c>
       <c r="N178" t="s" s="2">
-        <v>113</v>
+        <v>831</v>
       </c>
       <c r="O178" s="2"/>
       <c r="P178" t="s" s="2">
@@ -24132,19 +23899,19 @@
         <v>79</v>
       </c>
       <c r="AB178" t="s" s="2">
-        <v>114</v>
+        <v>79</v>
       </c>
       <c r="AC178" t="s" s="2">
-        <v>115</v>
+        <v>79</v>
       </c>
       <c r="AD178" t="s" s="2">
         <v>79</v>
       </c>
       <c r="AE178" t="s" s="2">
-        <v>116</v>
+        <v>79</v>
       </c>
       <c r="AF178" t="s" s="2">
-        <v>117</v>
+        <v>826</v>
       </c>
       <c r="AG178" t="s" s="2">
         <v>77</v>
@@ -24156,19 +23923,19 @@
         <v>99</v>
       </c>
       <c r="AJ178" t="s" s="2">
-        <v>118</v>
+        <v>481</v>
       </c>
       <c r="AK178" t="s" s="2">
-        <v>101</v>
+        <v>832</v>
       </c>
       <c r="AL178" t="s" s="2">
-        <v>79</v>
+        <v>107</v>
       </c>
       <c r="AM178" t="s" s="2">
         <v>79</v>
       </c>
       <c r="AN178" t="s" s="2">
-        <v>79</v>
+        <v>833</v>
       </c>
       <c r="AO178" t="s" s="2">
         <v>79</v>
@@ -24176,10 +23943,10 @@
     </row>
     <row r="179">
       <c r="A179" t="s" s="2">
-        <v>835</v>
+        <v>834</v>
       </c>
       <c r="B179" t="s" s="2">
-        <v>765</v>
+        <v>834</v>
       </c>
       <c r="C179" s="2"/>
       <c r="D179" t="s" s="2">
@@ -24190,7 +23957,7 @@
         <v>77</v>
       </c>
       <c r="G179" t="s" s="2">
-        <v>78</v>
+        <v>87</v>
       </c>
       <c r="H179" t="s" s="2">
         <v>79</v>
@@ -24202,19 +23969,19 @@
         <v>88</v>
       </c>
       <c r="K179" t="s" s="2">
-        <v>147</v>
+        <v>835</v>
       </c>
       <c r="L179" t="s" s="2">
-        <v>766</v>
+        <v>836</v>
       </c>
       <c r="M179" t="s" s="2">
-        <v>767</v>
+        <v>837</v>
       </c>
       <c r="N179" t="s" s="2">
-        <v>768</v>
+        <v>838</v>
       </c>
       <c r="O179" t="s" s="2">
-        <v>769</v>
+        <v>839</v>
       </c>
       <c r="P179" t="s" s="2">
         <v>79</v>
@@ -24263,31 +24030,31 @@
         <v>79</v>
       </c>
       <c r="AF179" t="s" s="2">
-        <v>770</v>
+        <v>834</v>
       </c>
       <c r="AG179" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AH179" t="s" s="2">
-        <v>78</v>
+        <v>87</v>
       </c>
       <c r="AI179" t="s" s="2">
         <v>99</v>
       </c>
       <c r="AJ179" t="s" s="2">
-        <v>100</v>
+        <v>481</v>
       </c>
       <c r="AK179" t="s" s="2">
-        <v>771</v>
+        <v>793</v>
       </c>
       <c r="AL179" t="s" s="2">
-        <v>79</v>
+        <v>840</v>
       </c>
       <c r="AM179" t="s" s="2">
         <v>79</v>
       </c>
       <c r="AN179" t="s" s="2">
-        <v>772</v>
+        <v>79</v>
       </c>
       <c r="AO179" t="s" s="2">
         <v>79</v>
@@ -24295,10 +24062,10 @@
     </row>
     <row r="180">
       <c r="A180" t="s" s="2">
-        <v>836</v>
+        <v>841</v>
       </c>
       <c r="B180" t="s" s="2">
-        <v>774</v>
+        <v>841</v>
       </c>
       <c r="C180" s="2"/>
       <c r="D180" t="s" s="2">
@@ -24309,28 +24076,32 @@
         <v>77</v>
       </c>
       <c r="G180" t="s" s="2">
-        <v>87</v>
+        <v>78</v>
       </c>
       <c r="H180" t="s" s="2">
         <v>79</v>
       </c>
       <c r="I180" t="s" s="2">
-        <v>79</v>
+        <v>88</v>
       </c>
       <c r="J180" t="s" s="2">
-        <v>79</v>
+        <v>88</v>
       </c>
       <c r="K180" t="s" s="2">
-        <v>103</v>
+        <v>723</v>
       </c>
       <c r="L180" t="s" s="2">
-        <v>104</v>
+        <v>842</v>
       </c>
       <c r="M180" t="s" s="2">
-        <v>105</v>
-      </c>
-      <c r="N180" s="2"/>
-      <c r="O180" s="2"/>
+        <v>843</v>
+      </c>
+      <c r="N180" t="s" s="2">
+        <v>844</v>
+      </c>
+      <c r="O180" t="s" s="2">
+        <v>845</v>
+      </c>
       <c r="P180" t="s" s="2">
         <v>79</v>
       </c>
@@ -24378,25 +24149,25 @@
         <v>79</v>
       </c>
       <c r="AF180" t="s" s="2">
-        <v>106</v>
+        <v>841</v>
       </c>
       <c r="AG180" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AH180" t="s" s="2">
-        <v>87</v>
+        <v>78</v>
       </c>
       <c r="AI180" t="s" s="2">
-        <v>79</v>
+        <v>99</v>
       </c>
       <c r="AJ180" t="s" s="2">
-        <v>79</v>
+        <v>100</v>
       </c>
       <c r="AK180" t="s" s="2">
+        <v>846</v>
+      </c>
+      <c r="AL180" t="s" s="2">
         <v>107</v>
-      </c>
-      <c r="AL180" t="s" s="2">
-        <v>79</v>
       </c>
       <c r="AM180" t="s" s="2">
         <v>79</v>
@@ -24410,21 +24181,21 @@
     </row>
     <row r="181">
       <c r="A181" t="s" s="2">
-        <v>837</v>
+        <v>847</v>
       </c>
       <c r="B181" t="s" s="2">
-        <v>776</v>
+        <v>847</v>
       </c>
       <c r="C181" s="2"/>
       <c r="D181" t="s" s="2">
-        <v>109</v>
+        <v>79</v>
       </c>
       <c r="E181" s="2"/>
       <c r="F181" t="s" s="2">
         <v>77</v>
       </c>
       <c r="G181" t="s" s="2">
-        <v>78</v>
+        <v>87</v>
       </c>
       <c r="H181" t="s" s="2">
         <v>79</v>
@@ -24436,17 +24207,15 @@
         <v>79</v>
       </c>
       <c r="K181" t="s" s="2">
-        <v>110</v>
+        <v>103</v>
       </c>
       <c r="L181" t="s" s="2">
-        <v>111</v>
+        <v>104</v>
       </c>
       <c r="M181" t="s" s="2">
-        <v>112</v>
-      </c>
-      <c r="N181" t="s" s="2">
-        <v>113</v>
-      </c>
+        <v>105</v>
+      </c>
+      <c r="N181" s="2"/>
       <c r="O181" s="2"/>
       <c r="P181" t="s" s="2">
         <v>79</v>
@@ -24483,34 +24252,34 @@
         <v>79</v>
       </c>
       <c r="AB181" t="s" s="2">
-        <v>114</v>
+        <v>79</v>
       </c>
       <c r="AC181" t="s" s="2">
-        <v>115</v>
+        <v>79</v>
       </c>
       <c r="AD181" t="s" s="2">
         <v>79</v>
       </c>
       <c r="AE181" t="s" s="2">
-        <v>116</v>
+        <v>79</v>
       </c>
       <c r="AF181" t="s" s="2">
-        <v>117</v>
+        <v>106</v>
       </c>
       <c r="AG181" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AH181" t="s" s="2">
-        <v>78</v>
+        <v>87</v>
       </c>
       <c r="AI181" t="s" s="2">
-        <v>99</v>
+        <v>79</v>
       </c>
       <c r="AJ181" t="s" s="2">
-        <v>118</v>
+        <v>79</v>
       </c>
       <c r="AK181" t="s" s="2">
-        <v>101</v>
+        <v>107</v>
       </c>
       <c r="AL181" t="s" s="2">
         <v>79</v>
@@ -24527,21 +24296,21 @@
     </row>
     <row r="182">
       <c r="A182" t="s" s="2">
-        <v>838</v>
+        <v>848</v>
       </c>
       <c r="B182" t="s" s="2">
-        <v>778</v>
+        <v>848</v>
       </c>
       <c r="C182" s="2"/>
       <c r="D182" t="s" s="2">
-        <v>79</v>
+        <v>109</v>
       </c>
       <c r="E182" s="2"/>
       <c r="F182" t="s" s="2">
-        <v>87</v>
+        <v>77</v>
       </c>
       <c r="G182" t="s" s="2">
-        <v>87</v>
+        <v>78</v>
       </c>
       <c r="H182" t="s" s="2">
         <v>79</v>
@@ -24550,23 +24319,21 @@
         <v>79</v>
       </c>
       <c r="J182" t="s" s="2">
-        <v>88</v>
+        <v>79</v>
       </c>
       <c r="K182" t="s" s="2">
-        <v>131</v>
+        <v>110</v>
       </c>
       <c r="L182" t="s" s="2">
-        <v>779</v>
+        <v>111</v>
       </c>
       <c r="M182" t="s" s="2">
-        <v>780</v>
+        <v>112</v>
       </c>
       <c r="N182" t="s" s="2">
-        <v>781</v>
-      </c>
-      <c r="O182" t="s" s="2">
-        <v>782</v>
-      </c>
+        <v>113</v>
+      </c>
+      <c r="O182" s="2"/>
       <c r="P182" t="s" s="2">
         <v>79</v>
       </c>
@@ -24575,7 +24342,7 @@
         <v>79</v>
       </c>
       <c r="S182" t="s" s="2">
-        <v>839</v>
+        <v>79</v>
       </c>
       <c r="T182" t="s" s="2">
         <v>79</v>
@@ -24602,34 +24369,34 @@
         <v>79</v>
       </c>
       <c r="AB182" t="s" s="2">
-        <v>79</v>
+        <v>114</v>
       </c>
       <c r="AC182" t="s" s="2">
-        <v>79</v>
+        <v>115</v>
       </c>
       <c r="AD182" t="s" s="2">
         <v>79</v>
       </c>
       <c r="AE182" t="s" s="2">
-        <v>79</v>
+        <v>116</v>
       </c>
       <c r="AF182" t="s" s="2">
-        <v>784</v>
+        <v>117</v>
       </c>
       <c r="AG182" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AH182" t="s" s="2">
-        <v>87</v>
+        <v>78</v>
       </c>
       <c r="AI182" t="s" s="2">
         <v>99</v>
       </c>
       <c r="AJ182" t="s" s="2">
-        <v>100</v>
+        <v>118</v>
       </c>
       <c r="AK182" t="s" s="2">
-        <v>785</v>
+        <v>101</v>
       </c>
       <c r="AL182" t="s" s="2">
         <v>79</v>
@@ -24638,7 +24405,7 @@
         <v>79</v>
       </c>
       <c r="AN182" t="s" s="2">
-        <v>786</v>
+        <v>79</v>
       </c>
       <c r="AO182" t="s" s="2">
         <v>79</v>
@@ -24646,44 +24413,46 @@
     </row>
     <row r="183">
       <c r="A183" t="s" s="2">
-        <v>840</v>
+        <v>849</v>
       </c>
       <c r="B183" t="s" s="2">
-        <v>788</v>
+        <v>849</v>
       </c>
       <c r="C183" s="2"/>
       <c r="D183" t="s" s="2">
-        <v>79</v>
+        <v>743</v>
       </c>
       <c r="E183" s="2"/>
       <c r="F183" t="s" s="2">
         <v>77</v>
       </c>
       <c r="G183" t="s" s="2">
-        <v>87</v>
+        <v>78</v>
       </c>
       <c r="H183" t="s" s="2">
         <v>79</v>
       </c>
       <c r="I183" t="s" s="2">
-        <v>79</v>
+        <v>88</v>
       </c>
       <c r="J183" t="s" s="2">
         <v>88</v>
       </c>
       <c r="K183" t="s" s="2">
-        <v>103</v>
+        <v>110</v>
       </c>
       <c r="L183" t="s" s="2">
-        <v>789</v>
+        <v>744</v>
       </c>
       <c r="M183" t="s" s="2">
-        <v>790</v>
+        <v>745</v>
       </c>
       <c r="N183" t="s" s="2">
-        <v>791</v>
-      </c>
-      <c r="O183" s="2"/>
+        <v>113</v>
+      </c>
+      <c r="O183" t="s" s="2">
+        <v>404</v>
+      </c>
       <c r="P183" t="s" s="2">
         <v>79</v>
       </c>
@@ -24731,22 +24500,22 @@
         <v>79</v>
       </c>
       <c r="AF183" t="s" s="2">
-        <v>792</v>
+        <v>746</v>
       </c>
       <c r="AG183" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AH183" t="s" s="2">
-        <v>87</v>
+        <v>78</v>
       </c>
       <c r="AI183" t="s" s="2">
         <v>99</v>
       </c>
       <c r="AJ183" t="s" s="2">
-        <v>100</v>
+        <v>118</v>
       </c>
       <c r="AK183" t="s" s="2">
-        <v>793</v>
+        <v>101</v>
       </c>
       <c r="AL183" t="s" s="2">
         <v>79</v>
@@ -24755,7 +24524,7 @@
         <v>79</v>
       </c>
       <c r="AN183" t="s" s="2">
-        <v>794</v>
+        <v>79</v>
       </c>
       <c r="AO183" t="s" s="2">
         <v>79</v>
@@ -24763,10 +24532,10 @@
     </row>
     <row r="184">
       <c r="A184" t="s" s="2">
-        <v>841</v>
+        <v>850</v>
       </c>
       <c r="B184" t="s" s="2">
-        <v>796</v>
+        <v>850</v>
       </c>
       <c r="C184" s="2"/>
       <c r="D184" t="s" s="2">
@@ -24774,7 +24543,7 @@
       </c>
       <c r="E184" s="2"/>
       <c r="F184" t="s" s="2">
-        <v>77</v>
+        <v>87</v>
       </c>
       <c r="G184" t="s" s="2">
         <v>87</v>
@@ -24789,20 +24558,18 @@
         <v>88</v>
       </c>
       <c r="K184" t="s" s="2">
-        <v>171</v>
+        <v>851</v>
       </c>
       <c r="L184" t="s" s="2">
-        <v>797</v>
+        <v>852</v>
       </c>
       <c r="M184" t="s" s="2">
-        <v>798</v>
+        <v>853</v>
       </c>
       <c r="N184" t="s" s="2">
-        <v>340</v>
-      </c>
-      <c r="O184" t="s" s="2">
-        <v>799</v>
-      </c>
+        <v>854</v>
+      </c>
+      <c r="O184" s="2"/>
       <c r="P184" t="s" s="2">
         <v>79</v>
       </c>
@@ -24850,10 +24617,10 @@
         <v>79</v>
       </c>
       <c r="AF184" t="s" s="2">
-        <v>800</v>
+        <v>850</v>
       </c>
       <c r="AG184" t="s" s="2">
-        <v>77</v>
+        <v>87</v>
       </c>
       <c r="AH184" t="s" s="2">
         <v>87</v>
@@ -24862,19 +24629,19 @@
         <v>99</v>
       </c>
       <c r="AJ184" t="s" s="2">
-        <v>100</v>
+        <v>481</v>
       </c>
       <c r="AK184" t="s" s="2">
-        <v>801</v>
+        <v>413</v>
       </c>
       <c r="AL184" t="s" s="2">
-        <v>79</v>
+        <v>107</v>
       </c>
       <c r="AM184" t="s" s="2">
         <v>79</v>
       </c>
       <c r="AN184" t="s" s="2">
-        <v>802</v>
+        <v>855</v>
       </c>
       <c r="AO184" t="s" s="2">
         <v>79</v>
@@ -24882,10 +24649,10 @@
     </row>
     <row r="185">
       <c r="A185" t="s" s="2">
-        <v>842</v>
+        <v>856</v>
       </c>
       <c r="B185" t="s" s="2">
-        <v>804</v>
+        <v>856</v>
       </c>
       <c r="C185" s="2"/>
       <c r="D185" t="s" s="2">
@@ -24893,7 +24660,7 @@
       </c>
       <c r="E185" s="2"/>
       <c r="F185" t="s" s="2">
-        <v>77</v>
+        <v>87</v>
       </c>
       <c r="G185" t="s" s="2">
         <v>87</v>
@@ -24908,20 +24675,18 @@
         <v>88</v>
       </c>
       <c r="K185" t="s" s="2">
-        <v>103</v>
+        <v>171</v>
       </c>
       <c r="L185" t="s" s="2">
-        <v>805</v>
+        <v>857</v>
       </c>
       <c r="M185" t="s" s="2">
-        <v>806</v>
+        <v>858</v>
       </c>
       <c r="N185" t="s" s="2">
         <v>340</v>
       </c>
-      <c r="O185" t="s" s="2">
-        <v>807</v>
-      </c>
+      <c r="O185" s="2"/>
       <c r="P185" t="s" s="2">
         <v>79</v>
       </c>
@@ -24945,13 +24710,13 @@
         <v>79</v>
       </c>
       <c r="X185" t="s" s="2">
-        <v>79</v>
+        <v>262</v>
       </c>
       <c r="Y185" t="s" s="2">
-        <v>79</v>
+        <v>858</v>
       </c>
       <c r="Z185" t="s" s="2">
-        <v>79</v>
+        <v>859</v>
       </c>
       <c r="AA185" t="s" s="2">
         <v>79</v>
@@ -24969,10 +24734,10 @@
         <v>79</v>
       </c>
       <c r="AF185" t="s" s="2">
-        <v>808</v>
+        <v>856</v>
       </c>
       <c r="AG185" t="s" s="2">
-        <v>77</v>
+        <v>87</v>
       </c>
       <c r="AH185" t="s" s="2">
         <v>87</v>
@@ -24984,2616 +24749,18 @@
         <v>100</v>
       </c>
       <c r="AK185" t="s" s="2">
-        <v>809</v>
+        <v>860</v>
       </c>
       <c r="AL185" t="s" s="2">
-        <v>79</v>
+        <v>107</v>
       </c>
       <c r="AM185" t="s" s="2">
         <v>79</v>
       </c>
       <c r="AN185" t="s" s="2">
-        <v>810</v>
+        <v>79</v>
       </c>
       <c r="AO185" t="s" s="2">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="186">
-      <c r="A186" t="s" s="2">
-        <v>843</v>
-      </c>
-      <c r="B186" t="s" s="2">
-        <v>812</v>
-      </c>
-      <c r="C186" s="2"/>
-      <c r="D186" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="E186" s="2"/>
-      <c r="F186" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="G186" t="s" s="2">
-        <v>87</v>
-      </c>
-      <c r="H186" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="I186" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="J186" t="s" s="2">
-        <v>88</v>
-      </c>
-      <c r="K186" t="s" s="2">
-        <v>557</v>
-      </c>
-      <c r="L186" t="s" s="2">
-        <v>813</v>
-      </c>
-      <c r="M186" t="s" s="2">
-        <v>814</v>
-      </c>
-      <c r="N186" t="s" s="2">
-        <v>815</v>
-      </c>
-      <c r="O186" t="s" s="2">
-        <v>816</v>
-      </c>
-      <c r="P186" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="Q186" s="2"/>
-      <c r="R186" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="S186" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="T186" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="U186" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="V186" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="W186" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="X186" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="Y186" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="Z186" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AA186" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AB186" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AC186" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AD186" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AE186" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AF186" t="s" s="2">
-        <v>817</v>
-      </c>
-      <c r="AG186" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AH186" t="s" s="2">
-        <v>87</v>
-      </c>
-      <c r="AI186" t="s" s="2">
-        <v>99</v>
-      </c>
-      <c r="AJ186" t="s" s="2">
-        <v>100</v>
-      </c>
-      <c r="AK186" t="s" s="2">
-        <v>818</v>
-      </c>
-      <c r="AL186" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AM186" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AN186" t="s" s="2">
-        <v>819</v>
-      </c>
-      <c r="AO186" t="s" s="2">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="187">
-      <c r="A187" t="s" s="2">
-        <v>844</v>
-      </c>
-      <c r="B187" t="s" s="2">
-        <v>821</v>
-      </c>
-      <c r="C187" s="2"/>
-      <c r="D187" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="E187" s="2"/>
-      <c r="F187" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="G187" t="s" s="2">
-        <v>87</v>
-      </c>
-      <c r="H187" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="I187" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="J187" t="s" s="2">
-        <v>88</v>
-      </c>
-      <c r="K187" t="s" s="2">
-        <v>103</v>
-      </c>
-      <c r="L187" t="s" s="2">
-        <v>822</v>
-      </c>
-      <c r="M187" t="s" s="2">
-        <v>823</v>
-      </c>
-      <c r="N187" t="s" s="2">
-        <v>824</v>
-      </c>
-      <c r="O187" t="s" s="2">
-        <v>825</v>
-      </c>
-      <c r="P187" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="Q187" s="2"/>
-      <c r="R187" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="S187" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="T187" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="U187" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="V187" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="W187" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="X187" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="Y187" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="Z187" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AA187" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AB187" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AC187" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AD187" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AE187" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AF187" t="s" s="2">
-        <v>826</v>
-      </c>
-      <c r="AG187" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AH187" t="s" s="2">
-        <v>87</v>
-      </c>
-      <c r="AI187" t="s" s="2">
-        <v>99</v>
-      </c>
-      <c r="AJ187" t="s" s="2">
-        <v>100</v>
-      </c>
-      <c r="AK187" t="s" s="2">
-        <v>827</v>
-      </c>
-      <c r="AL187" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AM187" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AN187" t="s" s="2">
-        <v>828</v>
-      </c>
-      <c r="AO187" t="s" s="2">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="188">
-      <c r="A188" t="s" s="2">
-        <v>845</v>
-      </c>
-      <c r="B188" t="s" s="2">
-        <v>845</v>
-      </c>
-      <c r="C188" s="2"/>
-      <c r="D188" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="E188" s="2"/>
-      <c r="F188" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="G188" t="s" s="2">
-        <v>87</v>
-      </c>
-      <c r="H188" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="I188" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="J188" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="K188" t="s" s="2">
-        <v>566</v>
-      </c>
-      <c r="L188" t="s" s="2">
-        <v>846</v>
-      </c>
-      <c r="M188" t="s" s="2">
-        <v>847</v>
-      </c>
-      <c r="N188" t="s" s="2">
-        <v>848</v>
-      </c>
-      <c r="O188" t="s" s="2">
-        <v>849</v>
-      </c>
-      <c r="P188" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="Q188" s="2"/>
-      <c r="R188" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="S188" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="T188" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="U188" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="V188" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="W188" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="X188" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="Y188" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="Z188" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AA188" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AB188" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AC188" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AD188" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AE188" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AF188" t="s" s="2">
-        <v>845</v>
-      </c>
-      <c r="AG188" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AH188" t="s" s="2">
-        <v>87</v>
-      </c>
-      <c r="AI188" t="s" s="2">
-        <v>99</v>
-      </c>
-      <c r="AJ188" t="s" s="2">
-        <v>100</v>
-      </c>
-      <c r="AK188" t="s" s="2">
-        <v>850</v>
-      </c>
-      <c r="AL188" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AM188" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AN188" t="s" s="2">
-        <v>851</v>
-      </c>
-      <c r="AO188" t="s" s="2">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="189">
-      <c r="A189" t="s" s="2">
-        <v>852</v>
-      </c>
-      <c r="B189" t="s" s="2">
-        <v>852</v>
-      </c>
-      <c r="C189" s="2"/>
-      <c r="D189" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="E189" s="2"/>
-      <c r="F189" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="G189" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="H189" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="I189" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="J189" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="K189" t="s" s="2">
-        <v>660</v>
-      </c>
-      <c r="L189" t="s" s="2">
-        <v>661</v>
-      </c>
-      <c r="M189" t="s" s="2">
-        <v>662</v>
-      </c>
-      <c r="N189" t="s" s="2">
-        <v>853</v>
-      </c>
-      <c r="O189" t="s" s="2">
-        <v>664</v>
-      </c>
-      <c r="P189" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="Q189" s="2"/>
-      <c r="R189" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="S189" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="T189" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="U189" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="V189" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="W189" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="X189" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="Y189" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="Z189" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AA189" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AB189" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AC189" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AD189" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AE189" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AF189" t="s" s="2">
-        <v>852</v>
-      </c>
-      <c r="AG189" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AH189" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AI189" t="s" s="2">
-        <v>99</v>
-      </c>
-      <c r="AJ189" t="s" s="2">
-        <v>665</v>
-      </c>
-      <c r="AK189" t="s" s="2">
-        <v>666</v>
-      </c>
-      <c r="AL189" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AM189" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AN189" t="s" s="2">
-        <v>667</v>
-      </c>
-      <c r="AO189" t="s" s="2">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="190">
-      <c r="A190" t="s" s="2">
-        <v>854</v>
-      </c>
-      <c r="B190" t="s" s="2">
-        <v>854</v>
-      </c>
-      <c r="C190" s="2"/>
-      <c r="D190" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="E190" s="2"/>
-      <c r="F190" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="G190" t="s" s="2">
-        <v>87</v>
-      </c>
-      <c r="H190" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="I190" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="J190" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="K190" t="s" s="2">
-        <v>855</v>
-      </c>
-      <c r="L190" t="s" s="2">
-        <v>856</v>
-      </c>
-      <c r="M190" t="s" s="2">
-        <v>857</v>
-      </c>
-      <c r="N190" t="s" s="2">
-        <v>292</v>
-      </c>
-      <c r="O190" t="s" s="2">
-        <v>858</v>
-      </c>
-      <c r="P190" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="Q190" s="2"/>
-      <c r="R190" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="S190" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="T190" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="U190" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="V190" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="W190" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="X190" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="Y190" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="Z190" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AA190" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AB190" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AC190" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AD190" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AE190" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AF190" t="s" s="2">
-        <v>854</v>
-      </c>
-      <c r="AG190" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AH190" t="s" s="2">
-        <v>87</v>
-      </c>
-      <c r="AI190" t="s" s="2">
-        <v>99</v>
-      </c>
-      <c r="AJ190" t="s" s="2">
-        <v>100</v>
-      </c>
-      <c r="AK190" t="s" s="2">
-        <v>859</v>
-      </c>
-      <c r="AL190" t="s" s="2">
-        <v>107</v>
-      </c>
-      <c r="AM190" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AN190" t="s" s="2">
-        <v>860</v>
-      </c>
-      <c r="AO190" t="s" s="2">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="191">
-      <c r="A191" t="s" s="2">
-        <v>861</v>
-      </c>
-      <c r="B191" t="s" s="2">
-        <v>861</v>
-      </c>
-      <c r="C191" s="2"/>
-      <c r="D191" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="E191" s="2"/>
-      <c r="F191" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="G191" t="s" s="2">
-        <v>87</v>
-      </c>
-      <c r="H191" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="I191" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="J191" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="K191" t="s" s="2">
-        <v>171</v>
-      </c>
-      <c r="L191" t="s" s="2">
-        <v>862</v>
-      </c>
-      <c r="M191" t="s" s="2">
-        <v>863</v>
-      </c>
-      <c r="N191" t="s" s="2">
-        <v>340</v>
-      </c>
-      <c r="O191" t="s" s="2">
-        <v>864</v>
-      </c>
-      <c r="P191" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="Q191" s="2"/>
-      <c r="R191" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="S191" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="T191" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="U191" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="V191" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="W191" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="X191" t="s" s="2">
-        <v>262</v>
-      </c>
-      <c r="Y191" t="s" s="2">
-        <v>865</v>
-      </c>
-      <c r="Z191" t="s" s="2">
-        <v>866</v>
-      </c>
-      <c r="AA191" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AB191" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AC191" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AD191" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AE191" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AF191" t="s" s="2">
-        <v>861</v>
-      </c>
-      <c r="AG191" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AH191" t="s" s="2">
-        <v>87</v>
-      </c>
-      <c r="AI191" t="s" s="2">
-        <v>99</v>
-      </c>
-      <c r="AJ191" t="s" s="2">
-        <v>100</v>
-      </c>
-      <c r="AK191" t="s" s="2">
-        <v>674</v>
-      </c>
-      <c r="AL191" t="s" s="2">
-        <v>107</v>
-      </c>
-      <c r="AM191" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AN191" t="s" s="2">
-        <v>867</v>
-      </c>
-      <c r="AO191" t="s" s="2">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="192">
-      <c r="A192" t="s" s="2">
-        <v>868</v>
-      </c>
-      <c r="B192" t="s" s="2">
-        <v>868</v>
-      </c>
-      <c r="C192" s="2"/>
-      <c r="D192" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="E192" s="2"/>
-      <c r="F192" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="G192" t="s" s="2">
-        <v>87</v>
-      </c>
-      <c r="H192" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="I192" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="J192" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="K192" t="s" s="2">
-        <v>476</v>
-      </c>
-      <c r="L192" t="s" s="2">
-        <v>869</v>
-      </c>
-      <c r="M192" t="s" s="2">
-        <v>870</v>
-      </c>
-      <c r="N192" t="s" s="2">
-        <v>871</v>
-      </c>
-      <c r="O192" t="s" s="2">
-        <v>872</v>
-      </c>
-      <c r="P192" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="Q192" s="2"/>
-      <c r="R192" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="S192" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="T192" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="U192" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="V192" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="W192" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="X192" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="Y192" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="Z192" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AA192" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AB192" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AC192" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AD192" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AE192" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AF192" t="s" s="2">
-        <v>868</v>
-      </c>
-      <c r="AG192" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AH192" t="s" s="2">
-        <v>87</v>
-      </c>
-      <c r="AI192" t="s" s="2">
-        <v>873</v>
-      </c>
-      <c r="AJ192" t="s" s="2">
-        <v>481</v>
-      </c>
-      <c r="AK192" t="s" s="2">
-        <v>874</v>
-      </c>
-      <c r="AL192" t="s" s="2">
-        <v>107</v>
-      </c>
-      <c r="AM192" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AN192" t="s" s="2">
-        <v>875</v>
-      </c>
-      <c r="AO192" t="s" s="2">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="193">
-      <c r="A193" t="s" s="2">
-        <v>876</v>
-      </c>
-      <c r="B193" t="s" s="2">
-        <v>876</v>
-      </c>
-      <c r="C193" s="2"/>
-      <c r="D193" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="E193" s="2"/>
-      <c r="F193" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="G193" t="s" s="2">
-        <v>87</v>
-      </c>
-      <c r="H193" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="I193" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="J193" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="K193" t="s" s="2">
-        <v>391</v>
-      </c>
-      <c r="L193" t="s" s="2">
-        <v>877</v>
-      </c>
-      <c r="M193" t="s" s="2">
-        <v>878</v>
-      </c>
-      <c r="N193" t="s" s="2">
-        <v>394</v>
-      </c>
-      <c r="O193" s="2"/>
-      <c r="P193" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="Q193" s="2"/>
-      <c r="R193" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="S193" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="T193" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="U193" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="V193" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="W193" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="X193" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="Y193" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="Z193" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AA193" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AB193" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AC193" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AD193" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AE193" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AF193" t="s" s="2">
-        <v>876</v>
-      </c>
-      <c r="AG193" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AH193" t="s" s="2">
-        <v>87</v>
-      </c>
-      <c r="AI193" t="s" s="2">
-        <v>99</v>
-      </c>
-      <c r="AJ193" t="s" s="2">
-        <v>398</v>
-      </c>
-      <c r="AK193" t="s" s="2">
-        <v>879</v>
-      </c>
-      <c r="AL193" t="s" s="2">
-        <v>107</v>
-      </c>
-      <c r="AM193" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AN193" t="s" s="2">
-        <v>880</v>
-      </c>
-      <c r="AO193" t="s" s="2">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="194">
-      <c r="A194" t="s" s="2">
-        <v>881</v>
-      </c>
-      <c r="B194" t="s" s="2">
-        <v>881</v>
-      </c>
-      <c r="C194" s="2"/>
-      <c r="D194" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="E194" s="2"/>
-      <c r="F194" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="G194" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="H194" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="I194" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="J194" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="K194" t="s" s="2">
-        <v>723</v>
-      </c>
-      <c r="L194" t="s" s="2">
-        <v>882</v>
-      </c>
-      <c r="M194" t="s" s="2">
-        <v>883</v>
-      </c>
-      <c r="N194" t="s" s="2">
-        <v>884</v>
-      </c>
-      <c r="O194" t="s" s="2">
-        <v>885</v>
-      </c>
-      <c r="P194" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="Q194" s="2"/>
-      <c r="R194" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="S194" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="T194" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="U194" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="V194" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="W194" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="X194" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="Y194" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="Z194" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AA194" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AB194" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AC194" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AD194" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AE194" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AF194" t="s" s="2">
-        <v>881</v>
-      </c>
-      <c r="AG194" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AH194" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AI194" t="s" s="2">
-        <v>99</v>
-      </c>
-      <c r="AJ194" t="s" s="2">
-        <v>100</v>
-      </c>
-      <c r="AK194" t="s" s="2">
-        <v>886</v>
-      </c>
-      <c r="AL194" t="s" s="2">
-        <v>887</v>
-      </c>
-      <c r="AM194" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AN194" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AO194" t="s" s="2">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="195">
-      <c r="A195" t="s" s="2">
-        <v>888</v>
-      </c>
-      <c r="B195" t="s" s="2">
-        <v>888</v>
-      </c>
-      <c r="C195" s="2"/>
-      <c r="D195" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="E195" s="2"/>
-      <c r="F195" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="G195" t="s" s="2">
-        <v>87</v>
-      </c>
-      <c r="H195" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="I195" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="J195" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="K195" t="s" s="2">
-        <v>103</v>
-      </c>
-      <c r="L195" t="s" s="2">
-        <v>104</v>
-      </c>
-      <c r="M195" t="s" s="2">
-        <v>105</v>
-      </c>
-      <c r="N195" s="2"/>
-      <c r="O195" s="2"/>
-      <c r="P195" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="Q195" s="2"/>
-      <c r="R195" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="S195" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="T195" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="U195" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="V195" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="W195" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="X195" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="Y195" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="Z195" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AA195" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AB195" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AC195" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AD195" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AE195" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AF195" t="s" s="2">
-        <v>106</v>
-      </c>
-      <c r="AG195" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AH195" t="s" s="2">
-        <v>87</v>
-      </c>
-      <c r="AI195" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AJ195" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AK195" t="s" s="2">
-        <v>107</v>
-      </c>
-      <c r="AL195" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AM195" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AN195" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AO195" t="s" s="2">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="196">
-      <c r="A196" t="s" s="2">
-        <v>889</v>
-      </c>
-      <c r="B196" t="s" s="2">
-        <v>889</v>
-      </c>
-      <c r="C196" s="2"/>
-      <c r="D196" t="s" s="2">
-        <v>109</v>
-      </c>
-      <c r="E196" s="2"/>
-      <c r="F196" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="G196" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="H196" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="I196" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="J196" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="K196" t="s" s="2">
-        <v>110</v>
-      </c>
-      <c r="L196" t="s" s="2">
-        <v>111</v>
-      </c>
-      <c r="M196" t="s" s="2">
-        <v>112</v>
-      </c>
-      <c r="N196" t="s" s="2">
-        <v>113</v>
-      </c>
-      <c r="O196" s="2"/>
-      <c r="P196" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="Q196" s="2"/>
-      <c r="R196" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="S196" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="T196" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="U196" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="V196" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="W196" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="X196" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="Y196" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="Z196" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AA196" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AB196" t="s" s="2">
-        <v>114</v>
-      </c>
-      <c r="AC196" t="s" s="2">
-        <v>115</v>
-      </c>
-      <c r="AD196" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AE196" t="s" s="2">
-        <v>116</v>
-      </c>
-      <c r="AF196" t="s" s="2">
-        <v>117</v>
-      </c>
-      <c r="AG196" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AH196" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AI196" t="s" s="2">
-        <v>99</v>
-      </c>
-      <c r="AJ196" t="s" s="2">
-        <v>118</v>
-      </c>
-      <c r="AK196" t="s" s="2">
-        <v>101</v>
-      </c>
-      <c r="AL196" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AM196" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AN196" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AO196" t="s" s="2">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="197">
-      <c r="A197" t="s" s="2">
-        <v>890</v>
-      </c>
-      <c r="B197" t="s" s="2">
-        <v>890</v>
-      </c>
-      <c r="C197" s="2"/>
-      <c r="D197" t="s" s="2">
-        <v>743</v>
-      </c>
-      <c r="E197" s="2"/>
-      <c r="F197" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="G197" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="H197" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="I197" t="s" s="2">
-        <v>88</v>
-      </c>
-      <c r="J197" t="s" s="2">
-        <v>88</v>
-      </c>
-      <c r="K197" t="s" s="2">
-        <v>110</v>
-      </c>
-      <c r="L197" t="s" s="2">
-        <v>744</v>
-      </c>
-      <c r="M197" t="s" s="2">
-        <v>745</v>
-      </c>
-      <c r="N197" t="s" s="2">
-        <v>113</v>
-      </c>
-      <c r="O197" t="s" s="2">
-        <v>404</v>
-      </c>
-      <c r="P197" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="Q197" s="2"/>
-      <c r="R197" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="S197" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="T197" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="U197" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="V197" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="W197" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="X197" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="Y197" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="Z197" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AA197" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AB197" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AC197" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AD197" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AE197" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AF197" t="s" s="2">
-        <v>746</v>
-      </c>
-      <c r="AG197" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AH197" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AI197" t="s" s="2">
-        <v>99</v>
-      </c>
-      <c r="AJ197" t="s" s="2">
-        <v>118</v>
-      </c>
-      <c r="AK197" t="s" s="2">
-        <v>101</v>
-      </c>
-      <c r="AL197" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AM197" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AN197" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AO197" t="s" s="2">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="198">
-      <c r="A198" t="s" s="2">
-        <v>891</v>
-      </c>
-      <c r="B198" t="s" s="2">
-        <v>891</v>
-      </c>
-      <c r="C198" s="2"/>
-      <c r="D198" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="E198" s="2"/>
-      <c r="F198" t="s" s="2">
-        <v>87</v>
-      </c>
-      <c r="G198" t="s" s="2">
-        <v>87</v>
-      </c>
-      <c r="H198" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="I198" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="J198" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="K198" t="s" s="2">
-        <v>438</v>
-      </c>
-      <c r="L198" t="s" s="2">
-        <v>892</v>
-      </c>
-      <c r="M198" t="s" s="2">
-        <v>893</v>
-      </c>
-      <c r="N198" t="s" s="2">
-        <v>894</v>
-      </c>
-      <c r="O198" t="s" s="2">
-        <v>895</v>
-      </c>
-      <c r="P198" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="Q198" s="2"/>
-      <c r="R198" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="S198" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="T198" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="U198" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="V198" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="W198" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="X198" t="s" s="2">
-        <v>175</v>
-      </c>
-      <c r="Y198" t="s" s="2">
-        <v>176</v>
-      </c>
-      <c r="Z198" t="s" s="2">
-        <v>177</v>
-      </c>
-      <c r="AA198" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AB198" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AC198" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AD198" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AE198" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AF198" t="s" s="2">
-        <v>891</v>
-      </c>
-      <c r="AG198" t="s" s="2">
-        <v>87</v>
-      </c>
-      <c r="AH198" t="s" s="2">
-        <v>87</v>
-      </c>
-      <c r="AI198" t="s" s="2">
-        <v>99</v>
-      </c>
-      <c r="AJ198" t="s" s="2">
-        <v>100</v>
-      </c>
-      <c r="AK198" t="s" s="2">
-        <v>896</v>
-      </c>
-      <c r="AL198" t="s" s="2">
-        <v>897</v>
-      </c>
-      <c r="AM198" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AN198" t="s" s="2">
-        <v>898</v>
-      </c>
-      <c r="AO198" t="s" s="2">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="199">
-      <c r="A199" t="s" s="2">
-        <v>899</v>
-      </c>
-      <c r="B199" t="s" s="2">
-        <v>899</v>
-      </c>
-      <c r="C199" s="2"/>
-      <c r="D199" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="E199" s="2"/>
-      <c r="F199" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="G199" t="s" s="2">
-        <v>87</v>
-      </c>
-      <c r="H199" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="I199" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="J199" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="K199" t="s" s="2">
-        <v>557</v>
-      </c>
-      <c r="L199" t="s" s="2">
-        <v>900</v>
-      </c>
-      <c r="M199" t="s" s="2">
-        <v>901</v>
-      </c>
-      <c r="N199" t="s" s="2">
-        <v>902</v>
-      </c>
-      <c r="O199" t="s" s="2">
-        <v>903</v>
-      </c>
-      <c r="P199" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="Q199" s="2"/>
-      <c r="R199" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="S199" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="T199" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="U199" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="V199" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="W199" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="X199" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="Y199" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="Z199" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AA199" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AB199" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AC199" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AD199" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AE199" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AF199" t="s" s="2">
-        <v>899</v>
-      </c>
-      <c r="AG199" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AH199" t="s" s="2">
-        <v>87</v>
-      </c>
-      <c r="AI199" t="s" s="2">
-        <v>99</v>
-      </c>
-      <c r="AJ199" t="s" s="2">
-        <v>100</v>
-      </c>
-      <c r="AK199" t="s" s="2">
-        <v>904</v>
-      </c>
-      <c r="AL199" t="s" s="2">
-        <v>905</v>
-      </c>
-      <c r="AM199" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AN199" t="s" s="2">
-        <v>906</v>
-      </c>
-      <c r="AO199" t="s" s="2">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="200">
-      <c r="A200" t="s" s="2">
-        <v>907</v>
-      </c>
-      <c r="B200" t="s" s="2">
-        <v>907</v>
-      </c>
-      <c r="C200" s="2"/>
-      <c r="D200" t="s" s="2">
-        <v>908</v>
-      </c>
-      <c r="E200" s="2"/>
-      <c r="F200" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="G200" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="H200" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="I200" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="J200" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="K200" t="s" s="2">
-        <v>909</v>
-      </c>
-      <c r="L200" t="s" s="2">
-        <v>910</v>
-      </c>
-      <c r="M200" t="s" s="2">
-        <v>911</v>
-      </c>
-      <c r="N200" t="s" s="2">
-        <v>912</v>
-      </c>
-      <c r="O200" s="2"/>
-      <c r="P200" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="Q200" s="2"/>
-      <c r="R200" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="S200" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="T200" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="U200" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="V200" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="W200" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="X200" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="Y200" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="Z200" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AA200" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AB200" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AC200" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AD200" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AE200" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AF200" t="s" s="2">
-        <v>907</v>
-      </c>
-      <c r="AG200" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AH200" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AI200" t="s" s="2">
-        <v>99</v>
-      </c>
-      <c r="AJ200" t="s" s="2">
-        <v>481</v>
-      </c>
-      <c r="AK200" t="s" s="2">
-        <v>913</v>
-      </c>
-      <c r="AL200" t="s" s="2">
-        <v>107</v>
-      </c>
-      <c r="AM200" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AN200" t="s" s="2">
-        <v>914</v>
-      </c>
-      <c r="AO200" t="s" s="2">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="201">
-      <c r="A201" t="s" s="2">
-        <v>915</v>
-      </c>
-      <c r="B201" t="s" s="2">
-        <v>915</v>
-      </c>
-      <c r="C201" s="2"/>
-      <c r="D201" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="E201" s="2"/>
-      <c r="F201" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="G201" t="s" s="2">
-        <v>87</v>
-      </c>
-      <c r="H201" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="I201" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="J201" t="s" s="2">
-        <v>88</v>
-      </c>
-      <c r="K201" t="s" s="2">
-        <v>916</v>
-      </c>
-      <c r="L201" t="s" s="2">
-        <v>917</v>
-      </c>
-      <c r="M201" t="s" s="2">
-        <v>918</v>
-      </c>
-      <c r="N201" t="s" s="2">
-        <v>919</v>
-      </c>
-      <c r="O201" t="s" s="2">
-        <v>920</v>
-      </c>
-      <c r="P201" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="Q201" s="2"/>
-      <c r="R201" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="S201" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="T201" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="U201" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="V201" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="W201" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="X201" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="Y201" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="Z201" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AA201" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AB201" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AC201" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AD201" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AE201" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AF201" t="s" s="2">
-        <v>915</v>
-      </c>
-      <c r="AG201" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AH201" t="s" s="2">
-        <v>87</v>
-      </c>
-      <c r="AI201" t="s" s="2">
-        <v>99</v>
-      </c>
-      <c r="AJ201" t="s" s="2">
-        <v>481</v>
-      </c>
-      <c r="AK201" t="s" s="2">
-        <v>874</v>
-      </c>
-      <c r="AL201" t="s" s="2">
-        <v>921</v>
-      </c>
-      <c r="AM201" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AN201" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AO201" t="s" s="2">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="202">
-      <c r="A202" t="s" s="2">
-        <v>922</v>
-      </c>
-      <c r="B202" t="s" s="2">
-        <v>922</v>
-      </c>
-      <c r="C202" s="2"/>
-      <c r="D202" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="E202" s="2"/>
-      <c r="F202" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="G202" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="H202" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="I202" t="s" s="2">
-        <v>88</v>
-      </c>
-      <c r="J202" t="s" s="2">
-        <v>88</v>
-      </c>
-      <c r="K202" t="s" s="2">
-        <v>723</v>
-      </c>
-      <c r="L202" t="s" s="2">
-        <v>923</v>
-      </c>
-      <c r="M202" t="s" s="2">
-        <v>924</v>
-      </c>
-      <c r="N202" t="s" s="2">
-        <v>925</v>
-      </c>
-      <c r="O202" t="s" s="2">
-        <v>926</v>
-      </c>
-      <c r="P202" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="Q202" s="2"/>
-      <c r="R202" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="S202" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="T202" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="U202" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="V202" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="W202" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="X202" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="Y202" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="Z202" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AA202" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AB202" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AC202" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AD202" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AE202" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AF202" t="s" s="2">
-        <v>922</v>
-      </c>
-      <c r="AG202" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AH202" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AI202" t="s" s="2">
-        <v>99</v>
-      </c>
-      <c r="AJ202" t="s" s="2">
-        <v>100</v>
-      </c>
-      <c r="AK202" t="s" s="2">
-        <v>927</v>
-      </c>
-      <c r="AL202" t="s" s="2">
-        <v>107</v>
-      </c>
-      <c r="AM202" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AN202" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AO202" t="s" s="2">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="203">
-      <c r="A203" t="s" s="2">
-        <v>928</v>
-      </c>
-      <c r="B203" t="s" s="2">
-        <v>928</v>
-      </c>
-      <c r="C203" s="2"/>
-      <c r="D203" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="E203" s="2"/>
-      <c r="F203" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="G203" t="s" s="2">
-        <v>87</v>
-      </c>
-      <c r="H203" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="I203" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="J203" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="K203" t="s" s="2">
-        <v>103</v>
-      </c>
-      <c r="L203" t="s" s="2">
-        <v>104</v>
-      </c>
-      <c r="M203" t="s" s="2">
-        <v>105</v>
-      </c>
-      <c r="N203" s="2"/>
-      <c r="O203" s="2"/>
-      <c r="P203" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="Q203" s="2"/>
-      <c r="R203" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="S203" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="T203" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="U203" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="V203" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="W203" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="X203" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="Y203" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="Z203" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AA203" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AB203" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AC203" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AD203" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AE203" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AF203" t="s" s="2">
-        <v>106</v>
-      </c>
-      <c r="AG203" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AH203" t="s" s="2">
-        <v>87</v>
-      </c>
-      <c r="AI203" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AJ203" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AK203" t="s" s="2">
-        <v>107</v>
-      </c>
-      <c r="AL203" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AM203" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AN203" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AO203" t="s" s="2">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="204">
-      <c r="A204" t="s" s="2">
-        <v>929</v>
-      </c>
-      <c r="B204" t="s" s="2">
-        <v>929</v>
-      </c>
-      <c r="C204" s="2"/>
-      <c r="D204" t="s" s="2">
-        <v>109</v>
-      </c>
-      <c r="E204" s="2"/>
-      <c r="F204" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="G204" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="H204" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="I204" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="J204" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="K204" t="s" s="2">
-        <v>110</v>
-      </c>
-      <c r="L204" t="s" s="2">
-        <v>111</v>
-      </c>
-      <c r="M204" t="s" s="2">
-        <v>112</v>
-      </c>
-      <c r="N204" t="s" s="2">
-        <v>113</v>
-      </c>
-      <c r="O204" s="2"/>
-      <c r="P204" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="Q204" s="2"/>
-      <c r="R204" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="S204" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="T204" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="U204" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="V204" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="W204" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="X204" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="Y204" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="Z204" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AA204" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AB204" t="s" s="2">
-        <v>114</v>
-      </c>
-      <c r="AC204" t="s" s="2">
-        <v>115</v>
-      </c>
-      <c r="AD204" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AE204" t="s" s="2">
-        <v>116</v>
-      </c>
-      <c r="AF204" t="s" s="2">
-        <v>117</v>
-      </c>
-      <c r="AG204" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AH204" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AI204" t="s" s="2">
-        <v>99</v>
-      </c>
-      <c r="AJ204" t="s" s="2">
-        <v>118</v>
-      </c>
-      <c r="AK204" t="s" s="2">
-        <v>101</v>
-      </c>
-      <c r="AL204" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AM204" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AN204" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AO204" t="s" s="2">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="205">
-      <c r="A205" t="s" s="2">
-        <v>930</v>
-      </c>
-      <c r="B205" t="s" s="2">
-        <v>930</v>
-      </c>
-      <c r="C205" s="2"/>
-      <c r="D205" t="s" s="2">
-        <v>743</v>
-      </c>
-      <c r="E205" s="2"/>
-      <c r="F205" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="G205" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="H205" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="I205" t="s" s="2">
-        <v>88</v>
-      </c>
-      <c r="J205" t="s" s="2">
-        <v>88</v>
-      </c>
-      <c r="K205" t="s" s="2">
-        <v>110</v>
-      </c>
-      <c r="L205" t="s" s="2">
-        <v>744</v>
-      </c>
-      <c r="M205" t="s" s="2">
-        <v>745</v>
-      </c>
-      <c r="N205" t="s" s="2">
-        <v>113</v>
-      </c>
-      <c r="O205" t="s" s="2">
-        <v>404</v>
-      </c>
-      <c r="P205" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="Q205" s="2"/>
-      <c r="R205" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="S205" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="T205" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="U205" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="V205" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="W205" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="X205" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="Y205" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="Z205" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AA205" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AB205" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AC205" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AD205" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AE205" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AF205" t="s" s="2">
-        <v>746</v>
-      </c>
-      <c r="AG205" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AH205" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AI205" t="s" s="2">
-        <v>99</v>
-      </c>
-      <c r="AJ205" t="s" s="2">
-        <v>118</v>
-      </c>
-      <c r="AK205" t="s" s="2">
-        <v>101</v>
-      </c>
-      <c r="AL205" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AM205" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AN205" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AO205" t="s" s="2">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="206">
-      <c r="A206" t="s" s="2">
-        <v>931</v>
-      </c>
-      <c r="B206" t="s" s="2">
-        <v>931</v>
-      </c>
-      <c r="C206" s="2"/>
-      <c r="D206" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="E206" s="2"/>
-      <c r="F206" t="s" s="2">
-        <v>87</v>
-      </c>
-      <c r="G206" t="s" s="2">
-        <v>87</v>
-      </c>
-      <c r="H206" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="I206" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="J206" t="s" s="2">
-        <v>88</v>
-      </c>
-      <c r="K206" t="s" s="2">
-        <v>932</v>
-      </c>
-      <c r="L206" t="s" s="2">
-        <v>933</v>
-      </c>
-      <c r="M206" t="s" s="2">
-        <v>934</v>
-      </c>
-      <c r="N206" t="s" s="2">
-        <v>935</v>
-      </c>
-      <c r="O206" s="2"/>
-      <c r="P206" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="Q206" s="2"/>
-      <c r="R206" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="S206" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="T206" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="U206" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="V206" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="W206" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="X206" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="Y206" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="Z206" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AA206" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AB206" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AC206" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AD206" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AE206" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AF206" t="s" s="2">
-        <v>931</v>
-      </c>
-      <c r="AG206" t="s" s="2">
-        <v>87</v>
-      </c>
-      <c r="AH206" t="s" s="2">
-        <v>87</v>
-      </c>
-      <c r="AI206" t="s" s="2">
-        <v>99</v>
-      </c>
-      <c r="AJ206" t="s" s="2">
-        <v>481</v>
-      </c>
-      <c r="AK206" t="s" s="2">
-        <v>413</v>
-      </c>
-      <c r="AL206" t="s" s="2">
-        <v>107</v>
-      </c>
-      <c r="AM206" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AN206" t="s" s="2">
-        <v>936</v>
-      </c>
-      <c r="AO206" t="s" s="2">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="207">
-      <c r="A207" t="s" s="2">
-        <v>937</v>
-      </c>
-      <c r="B207" t="s" s="2">
-        <v>937</v>
-      </c>
-      <c r="C207" s="2"/>
-      <c r="D207" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="E207" s="2"/>
-      <c r="F207" t="s" s="2">
-        <v>87</v>
-      </c>
-      <c r="G207" t="s" s="2">
-        <v>87</v>
-      </c>
-      <c r="H207" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="I207" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="J207" t="s" s="2">
-        <v>88</v>
-      </c>
-      <c r="K207" t="s" s="2">
-        <v>171</v>
-      </c>
-      <c r="L207" t="s" s="2">
-        <v>938</v>
-      </c>
-      <c r="M207" t="s" s="2">
-        <v>939</v>
-      </c>
-      <c r="N207" t="s" s="2">
-        <v>340</v>
-      </c>
-      <c r="O207" s="2"/>
-      <c r="P207" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="Q207" s="2"/>
-      <c r="R207" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="S207" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="T207" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="U207" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="V207" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="W207" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="X207" t="s" s="2">
-        <v>262</v>
-      </c>
-      <c r="Y207" t="s" s="2">
-        <v>939</v>
-      </c>
-      <c r="Z207" t="s" s="2">
-        <v>940</v>
-      </c>
-      <c r="AA207" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AB207" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AC207" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AD207" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AE207" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AF207" t="s" s="2">
-        <v>937</v>
-      </c>
-      <c r="AG207" t="s" s="2">
-        <v>87</v>
-      </c>
-      <c r="AH207" t="s" s="2">
-        <v>87</v>
-      </c>
-      <c r="AI207" t="s" s="2">
-        <v>99</v>
-      </c>
-      <c r="AJ207" t="s" s="2">
-        <v>100</v>
-      </c>
-      <c r="AK207" t="s" s="2">
-        <v>941</v>
-      </c>
-      <c r="AL207" t="s" s="2">
-        <v>107</v>
-      </c>
-      <c r="AM207" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AN207" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AO207" t="s" s="2">
         <v>79</v>
       </c>
     </row>

</xml_diff>